<commit_message>
nová verze s dlaždicemi
</commit_message>
<xml_diff>
--- a/data/Products.xlsx
+++ b/data/Products.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BA398"/>
+  <dimension ref="A1:BA392"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -57305,16 +57305,16 @@
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>TBD</v>
+        <v>Test01</v>
       </c>
       <c r="B391" t="str">
-        <v>TBD</v>
+        <v>357753</v>
       </c>
       <c r="C391" t="str">
         <v>Drylock</v>
       </c>
       <c r="D391" t="str">
-        <v>CZ11</v>
+        <v>CZ10</v>
       </c>
       <c r="E391" t="str">
         <v>CZ</v>
@@ -57323,49 +57323,49 @@
         <v>hygiene</v>
       </c>
       <c r="G391" t="str">
-        <v>TS</v>
+        <v>BEL</v>
       </c>
       <c r="H391" t="str">
         <v>S</v>
       </c>
       <c r="I391" t="str">
-        <v>bio Bico</v>
+        <v>Mono</v>
       </c>
       <c r="J391" t="str">
-        <v>G01 - Ovál</v>
+        <v>open dot</v>
       </c>
       <c r="K391" t="str">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="L391" t="str">
         <v/>
       </c>
       <c r="M391" t="str">
-        <v>hydrophilic</v>
+        <v/>
       </c>
       <c r="N391" t="str">
         <v>0 - natur</v>
       </c>
       <c r="O391" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P391" t="str">
-        <v>0.8207</v>
+        <v>Svobodová</v>
+      </c>
+      <c r="P391">
+        <v>0.8422</v>
       </c>
       <c r="Q391" t="str">
-        <v>1053</v>
+        <v>2768.8320000000003</v>
       </c>
       <c r="R391">
-        <v>1.1570245683958056</v>
+        <v>0.4288216447759506</v>
       </c>
       <c r="S391">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="T391">
-        <v>0</v>
+        <v>0.07</v>
       </c>
       <c r="U391">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="V391">
         <v>0.8</v>
@@ -57379,17 +57379,8 @@
       <c r="Y391">
         <v>0</v>
       </c>
-      <c r="Z391">
-        <v>0</v>
-      </c>
-      <c r="AA391">
-        <v>0.2</v>
-      </c>
-      <c r="AB391">
-        <v>0</v>
-      </c>
       <c r="AC391">
-        <v>0.007</v>
+        <v>0</v>
       </c>
       <c r="AD391">
         <v>0</v>
@@ -57413,7 +57404,7 @@
         <v>0</v>
       </c>
       <c r="AK391">
-        <v>1.007</v>
+        <v>1</v>
       </c>
       <c r="AL391" t="str">
         <v>S: PPSB - Mosten NB 425</v>
@@ -57427,17 +57418,8 @@
       <c r="AO391" t="str">
         <v/>
       </c>
-      <c r="AP391" t="str">
+      <c r="AS391" t="str">
         <v/>
-      </c>
-      <c r="AQ391" t="str">
-        <v>S: Bio HDPE SHA 7260</v>
-      </c>
-      <c r="AR391" t="str">
-        <v/>
-      </c>
-      <c r="AS391" t="str">
-        <v>S: Zušl. - Silastol PHP 90</v>
       </c>
       <c r="AT391" t="str">
         <v/>
@@ -57460,22 +57442,22 @@
       <c r="AZ391" t="str">
         <v/>
       </c>
-      <c r="BA391" t="str">
-        <v/>
+      <c r="BA391">
+        <v>0.03</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>Test01</v>
+        <v>New Test</v>
       </c>
       <c r="B392" t="str">
-        <v>357753</v>
+        <v>11111</v>
       </c>
       <c r="C392" t="str">
         <v>Drylock</v>
       </c>
       <c r="D392" t="str">
-        <v>CZ10</v>
+        <v>CZ05</v>
       </c>
       <c r="E392" t="str">
         <v>CZ</v>
@@ -57484,52 +57466,52 @@
         <v>hygiene</v>
       </c>
       <c r="G392" t="str">
-        <v>BEL</v>
+        <v>TS</v>
       </c>
       <c r="H392" t="str">
         <v>S</v>
       </c>
       <c r="I392" t="str">
-        <v>Mono</v>
+        <v>bio Bico</v>
       </c>
       <c r="J392" t="str">
-        <v>open dot</v>
+        <v>G01 - Ovál</v>
       </c>
       <c r="K392" t="str">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L392" t="str">
         <v/>
       </c>
       <c r="M392" t="str">
-        <v/>
+        <v>hydrophilic</v>
       </c>
       <c r="N392" t="str">
         <v>0 - natur</v>
       </c>
       <c r="O392" t="str">
-        <v>Svobodová</v>
+        <v>Svobodova</v>
       </c>
       <c r="P392">
-        <v>0.8422</v>
+        <v>0.7975</v>
       </c>
       <c r="Q392" t="str">
-        <v>2768.8320000000003</v>
+        <v>1538.9759999999994</v>
       </c>
       <c r="R392">
-        <v>0.4288216447759506</v>
+        <v>0.8147745613302652</v>
       </c>
       <c r="S392">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="T392">
-        <v>0.07</v>
+        <v>0.03</v>
       </c>
       <c r="U392">
-        <v>0.95</v>
+        <v>0.75</v>
       </c>
       <c r="V392">
-        <v>0.8</v>
+        <v>0.72</v>
       </c>
       <c r="W392">
         <v>0</v>
@@ -57540,8 +57522,14 @@
       <c r="Y392">
         <v>0</v>
       </c>
+      <c r="AA392">
+        <v>0.083</v>
+      </c>
+      <c r="AB392">
+        <v>0.166666</v>
+      </c>
       <c r="AC392">
-        <v>0</v>
+        <v>0.009</v>
       </c>
       <c r="AD392">
         <v>0</v>
@@ -57565,7 +57553,7 @@
         <v>0</v>
       </c>
       <c r="AK392">
-        <v>1</v>
+        <v>1.0086659999999998</v>
       </c>
       <c r="AL392" t="str">
         <v>S: PPSB - Mosten NB 425</v>
@@ -57579,8 +57567,14 @@
       <c r="AO392" t="str">
         <v/>
       </c>
+      <c r="AQ392" t="str">
+        <v>S: Bio HDPE SHA 7260</v>
+      </c>
+      <c r="AR392" t="str">
+        <v>S: PE Aspun 6850</v>
+      </c>
       <c r="AS392" t="str">
-        <v/>
+        <v>S: Zušl. - Silastol PHP 90</v>
       </c>
       <c r="AT392" t="str">
         <v/>
@@ -57604,945 +57598,12 @@
         <v/>
       </c>
       <c r="BA392">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" t="str">
-        <v>New Test</v>
-      </c>
-      <c r="B393" t="str">
-        <v>11111</v>
-      </c>
-      <c r="C393" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D393" t="str">
-        <v>CZ05</v>
-      </c>
-      <c r="E393" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F393" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G393" t="str">
-        <v>TS</v>
-      </c>
-      <c r="H393" t="str">
-        <v>S</v>
-      </c>
-      <c r="I393" t="str">
-        <v>bio Bico</v>
-      </c>
-      <c r="J393" t="str">
-        <v>G01 - Ovál</v>
-      </c>
-      <c r="K393" t="str">
-        <v>33</v>
-      </c>
-      <c r="L393" t="str">
-        <v/>
-      </c>
-      <c r="M393" t="str">
-        <v>hydrophilic</v>
-      </c>
-      <c r="N393" t="str">
-        <v>0 - natur</v>
-      </c>
-      <c r="O393" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P393">
-        <v>0.7975</v>
-      </c>
-      <c r="Q393" t="str">
-        <v>1538.9759999999994</v>
-      </c>
-      <c r="R393">
-        <v>0.8147745613302652</v>
-      </c>
-      <c r="S393">
-        <v>0</v>
-      </c>
-      <c r="T393">
-        <v>0.03</v>
-      </c>
-      <c r="U393">
-        <v>0.75</v>
-      </c>
-      <c r="V393">
-        <v>0.72</v>
-      </c>
-      <c r="W393">
-        <v>0</v>
-      </c>
-      <c r="X393">
-        <v>0</v>
-      </c>
-      <c r="Y393">
-        <v>0</v>
-      </c>
-      <c r="AA393">
-        <v>0.083</v>
-      </c>
-      <c r="AB393">
-        <v>0.166666</v>
-      </c>
-      <c r="AC393">
-        <v>0.009</v>
-      </c>
-      <c r="AD393">
-        <v>0</v>
-      </c>
-      <c r="AE393">
-        <v>0</v>
-      </c>
-      <c r="AF393">
-        <v>0</v>
-      </c>
-      <c r="AG393">
-        <v>0</v>
-      </c>
-      <c r="AH393">
-        <v>0</v>
-      </c>
-      <c r="AI393">
-        <v>0</v>
-      </c>
-      <c r="AJ393">
-        <v>0</v>
-      </c>
-      <c r="AK393">
-        <v>1.0086659999999998</v>
-      </c>
-      <c r="AL393" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM393" t="str">
-        <v/>
-      </c>
-      <c r="AN393" t="str">
-        <v/>
-      </c>
-      <c r="AO393" t="str">
-        <v/>
-      </c>
-      <c r="AQ393" t="str">
-        <v>S: Bio HDPE SHA 7260</v>
-      </c>
-      <c r="AR393" t="str">
-        <v>S: PE Aspun 6850</v>
-      </c>
-      <c r="AS393" t="str">
-        <v>S: Zušl. - Silastol PHP 90</v>
-      </c>
-      <c r="AT393" t="str">
-        <v/>
-      </c>
-      <c r="AU393" t="str">
-        <v/>
-      </c>
-      <c r="AV393" t="str">
-        <v/>
-      </c>
-      <c r="AW393" t="str">
-        <v/>
-      </c>
-      <c r="AX393" t="str">
-        <v/>
-      </c>
-      <c r="AY393" t="str">
-        <v/>
-      </c>
-      <c r="AZ393" t="str">
-        <v/>
-      </c>
-      <c r="BA393">
         <v>0.02</v>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" t="str">
-        <v/>
-      </c>
-      <c r="B394" t="str">
-        <v>1019 - testing edit</v>
-      </c>
-      <c r="C394" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D394" t="str">
-        <v>CZ11</v>
-      </c>
-      <c r="E394" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F394" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G394" t="str">
-        <v>BLC</v>
-      </c>
-      <c r="H394" t="str">
-        <v>SMS</v>
-      </c>
-      <c r="I394" t="str">
-        <v>Mono</v>
-      </c>
-      <c r="J394" t="str">
-        <v>G08 - honeycombs</v>
-      </c>
-      <c r="K394" t="str">
-        <v>14</v>
-      </c>
-      <c r="L394" t="str">
-        <v/>
-      </c>
-      <c r="M394" t="str">
-        <v>no treatment</v>
-      </c>
-      <c r="N394" t="str">
-        <v>100 - white</v>
-      </c>
-      <c r="O394" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P394">
-        <v>0.85</v>
-      </c>
-      <c r="Q394" t="str">
-        <v>1244</v>
-      </c>
-      <c r="R394">
-        <v>0.9457159069415548</v>
-      </c>
-      <c r="S394">
-        <v>0.08</v>
-      </c>
-      <c r="T394">
-        <v>0.08</v>
-      </c>
-      <c r="U394">
-        <v>0.8</v>
-      </c>
-      <c r="V394">
-        <v>0.6400000000000001</v>
-      </c>
-      <c r="W394">
-        <v>0.05</v>
-      </c>
-      <c r="X394">
-        <v>0</v>
-      </c>
-      <c r="Y394">
-        <v>0.143</v>
-      </c>
-      <c r="Z394">
-        <v>0</v>
-      </c>
-      <c r="AA394">
-        <v>0</v>
-      </c>
-      <c r="AB394">
-        <v>0</v>
-      </c>
-      <c r="AC394">
-        <v>0</v>
-      </c>
-      <c r="AD394">
-        <v>0</v>
-      </c>
-      <c r="AE394">
-        <v>0</v>
-      </c>
-      <c r="AF394">
-        <v>0.0024</v>
-      </c>
-      <c r="AG394">
-        <v>0</v>
-      </c>
-      <c r="AH394">
-        <v>0</v>
-      </c>
-      <c r="AI394">
-        <v>0.018</v>
-      </c>
-      <c r="AJ394">
-        <v>0</v>
-      </c>
-      <c r="AK394">
-        <v>0.9999999999999999</v>
-      </c>
-      <c r="AL394" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM394" t="str">
-        <v>S: PE Liten LS87</v>
-      </c>
-      <c r="AN394" t="str">
-        <v/>
-      </c>
-      <c r="AO394" t="str">
-        <v>S: PPMB - Borflow HL 708 FB</v>
-      </c>
-      <c r="AQ394" t="str">
-        <v/>
-      </c>
-      <c r="AS394" t="str">
-        <v/>
-      </c>
-      <c r="AT394" t="str">
-        <v/>
-      </c>
-      <c r="AU394" t="str">
-        <v/>
-      </c>
-      <c r="AV394" t="str">
-        <v>S: Pig.  - CC10084467BG b??l?? 60%</v>
-      </c>
-      <c r="AW394" t="str">
-        <v/>
-      </c>
-      <c r="AX394" t="str">
-        <v/>
-      </c>
-      <c r="AY394" t="str">
-        <v>S: Pig. - CC10098935BG slip ad. 10%Eruc.</v>
-      </c>
-      <c r="AZ394" t="str">
-        <v/>
-      </c>
-      <c r="BA394" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="B395" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="C395" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D395" t="str">
-        <v>CZ11</v>
-      </c>
-      <c r="E395" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F395" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G395" t="str">
-        <v>BLC</v>
-      </c>
-      <c r="H395" t="str">
-        <v>SMS</v>
-      </c>
-      <c r="I395" t="str">
-        <v>Mono</v>
-      </c>
-      <c r="J395" t="str">
-        <v>G08 - honeycombs</v>
-      </c>
-      <c r="K395">
-        <v>14</v>
-      </c>
-      <c r="L395">
-        <v>0</v>
-      </c>
-      <c r="M395" t="str">
-        <v>no treatment</v>
-      </c>
-      <c r="N395" t="str">
-        <v>100 - white</v>
-      </c>
-      <c r="O395" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P395">
-        <v>0.85</v>
-      </c>
-      <c r="Q395">
-        <v>1244</v>
-      </c>
-      <c r="R395">
-        <v>0.9457159069415548</v>
-      </c>
-      <c r="S395">
-        <v>0.08</v>
-      </c>
-      <c r="T395">
-        <v>0.08</v>
-      </c>
-      <c r="U395">
-        <v>0.85</v>
-      </c>
-      <c r="V395">
-        <v>0.6900000000000001</v>
-      </c>
-      <c r="W395">
-        <v>0</v>
-      </c>
-      <c r="X395">
-        <v>0</v>
-      </c>
-      <c r="Y395">
-        <v>0.143</v>
-      </c>
-      <c r="Z395">
-        <v>0</v>
-      </c>
-      <c r="AA395">
-        <v>0</v>
-      </c>
-      <c r="AB395">
-        <v>0</v>
-      </c>
-      <c r="AC395">
-        <v>0</v>
-      </c>
-      <c r="AD395">
-        <v>0</v>
-      </c>
-      <c r="AE395">
-        <v>0</v>
-      </c>
-      <c r="AF395">
-        <v>0.0024</v>
-      </c>
-      <c r="AG395">
-        <v>0</v>
-      </c>
-      <c r="AH395">
-        <v>0</v>
-      </c>
-      <c r="AI395">
-        <v>0.018</v>
-      </c>
-      <c r="AJ395">
-        <v>0</v>
-      </c>
-      <c r="AK395">
-        <v>0.9999999999999999</v>
-      </c>
-      <c r="AL395" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM395" t="str">
-        <v/>
-      </c>
-      <c r="AN395" t="str">
-        <v/>
-      </c>
-      <c r="AO395" t="str">
-        <v>S: PPMB - Borflow HL 708 FB</v>
-      </c>
-      <c r="AQ395" t="str">
-        <v/>
-      </c>
-      <c r="AS395" t="str">
-        <v/>
-      </c>
-      <c r="AT395" t="str">
-        <v/>
-      </c>
-      <c r="AU395" t="str">
-        <v/>
-      </c>
-      <c r="AV395" t="str">
-        <v>S: Pig.  - CC10084467BG b??l?? 60%</v>
-      </c>
-      <c r="AW395" t="str">
-        <v/>
-      </c>
-      <c r="AX395" t="str">
-        <v/>
-      </c>
-      <c r="AY395" t="str">
-        <v>S: Pig. - CC10098935BG slip ad. 10%Eruc.</v>
-      </c>
-      <c r="AZ395" t="str">
-        <v/>
-      </c>
-      <c r="BA395">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="B396" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="C396" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D396" t="str">
-        <v>CZ11</v>
-      </c>
-      <c r="E396" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F396" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G396" t="str">
-        <v>TS</v>
-      </c>
-      <c r="H396" t="str">
-        <v>S</v>
-      </c>
-      <c r="I396" t="str">
-        <v>bio Bico</v>
-      </c>
-      <c r="J396" t="str">
-        <v>G01 - Ovál</v>
-      </c>
-      <c r="K396" t="str">
-        <v>18</v>
-      </c>
-      <c r="L396" t="str">
-        <v/>
-      </c>
-      <c r="M396" t="str">
-        <v>hydrophilic</v>
-      </c>
-      <c r="N396" t="str">
-        <v>0 - natur</v>
-      </c>
-      <c r="O396" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P396">
-        <v>0.8207</v>
-      </c>
-      <c r="Q396" t="str">
-        <v>1053</v>
-      </c>
-      <c r="R396">
-        <v>1.1570245683958056</v>
-      </c>
-      <c r="S396">
-        <v>0</v>
-      </c>
-      <c r="T396">
-        <v>0</v>
-      </c>
-      <c r="U396">
-        <v>0.65</v>
-      </c>
-      <c r="V396">
-        <v>0.65</v>
-      </c>
-      <c r="W396">
-        <v>0</v>
-      </c>
-      <c r="X396">
-        <v>0</v>
-      </c>
-      <c r="Y396">
-        <v>0.15</v>
-      </c>
-      <c r="Z396">
-        <v>0</v>
-      </c>
-      <c r="AA396">
-        <v>0.2</v>
-      </c>
-      <c r="AB396">
-        <v>0</v>
-      </c>
-      <c r="AC396">
-        <v>0.007</v>
-      </c>
-      <c r="AD396">
-        <v>0</v>
-      </c>
-      <c r="AE396">
-        <v>0</v>
-      </c>
-      <c r="AF396">
-        <v>0</v>
-      </c>
-      <c r="AG396">
-        <v>0</v>
-      </c>
-      <c r="AH396">
-        <v>0</v>
-      </c>
-      <c r="AI396">
-        <v>0</v>
-      </c>
-      <c r="AJ396">
-        <v>0</v>
-      </c>
-      <c r="AK396">
-        <v>1.007</v>
-      </c>
-      <c r="AL396" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM396" t="str">
-        <v/>
-      </c>
-      <c r="AN396" t="str">
-        <v/>
-      </c>
-      <c r="AO396" t="str">
-        <v>S: PPMB - Borflow HL 712 FB</v>
-      </c>
-      <c r="AP396" t="str">
-        <v/>
-      </c>
-      <c r="AQ396" t="str">
-        <v>S: Bio HDPE SHA 7260</v>
-      </c>
-      <c r="AR396" t="str">
-        <v/>
-      </c>
-      <c r="AS396" t="str">
-        <v>S: Zušl. - Silastol PHP 90</v>
-      </c>
-      <c r="AT396" t="str">
-        <v/>
-      </c>
-      <c r="AU396" t="str">
-        <v/>
-      </c>
-      <c r="AV396" t="str">
-        <v/>
-      </c>
-      <c r="AW396" t="str">
-        <v/>
-      </c>
-      <c r="AX396" t="str">
-        <v/>
-      </c>
-      <c r="AY396" t="str">
-        <v/>
-      </c>
-      <c r="AZ396" t="str">
-        <v/>
-      </c>
-      <c r="BA396" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="B397" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="C397" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D397" t="str">
-        <v>CZ11</v>
-      </c>
-      <c r="E397" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F397" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G397" t="str">
-        <v>BS</v>
-      </c>
-      <c r="H397" t="str">
-        <v>S</v>
-      </c>
-      <c r="I397" t="str">
-        <v>bico</v>
-      </c>
-      <c r="J397" t="str">
-        <v>G01 - Ovál</v>
-      </c>
-      <c r="K397">
-        <v>12</v>
-      </c>
-      <c r="L397">
-        <v>0</v>
-      </c>
-      <c r="M397" t="str">
-        <v>no treatment</v>
-      </c>
-      <c r="N397" t="str">
-        <v>0 - natur</v>
-      </c>
-      <c r="O397" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P397">
-        <v>0.8473076923076923</v>
-      </c>
-      <c r="Q397">
-        <v>1169.28</v>
-      </c>
-      <c r="R397">
-        <v>1.0093466117383345</v>
-      </c>
-      <c r="S397">
-        <v>0</v>
-      </c>
-      <c r="T397">
-        <v>0.02</v>
-      </c>
-      <c r="U397">
-        <v>0.7</v>
-      </c>
-      <c r="V397">
-        <v>0.6799999999999999</v>
-      </c>
-      <c r="W397">
-        <v>0</v>
-      </c>
-      <c r="X397">
-        <v>0</v>
-      </c>
-      <c r="Y397">
-        <v>0</v>
-      </c>
-      <c r="Z397">
-        <v>0</v>
-      </c>
-      <c r="AA397">
-        <v>0.3</v>
-      </c>
-      <c r="AB397">
-        <v>0</v>
-      </c>
-      <c r="AC397">
-        <v>0</v>
-      </c>
-      <c r="AD397">
-        <v>0</v>
-      </c>
-      <c r="AE397">
-        <v>0</v>
-      </c>
-      <c r="AF397">
-        <v>0</v>
-      </c>
-      <c r="AG397">
-        <v>0</v>
-      </c>
-      <c r="AH397">
-        <v>0</v>
-      </c>
-      <c r="AI397">
-        <v>0</v>
-      </c>
-      <c r="AJ397">
-        <v>0</v>
-      </c>
-      <c r="AK397">
-        <v>1</v>
-      </c>
-      <c r="AL397" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM397" t="str">
-        <v>0</v>
-      </c>
-      <c r="AN397">
-        <v>0</v>
-      </c>
-      <c r="AO397">
-        <v>0</v>
-      </c>
-      <c r="AQ397" t="str">
-        <v>S: PE Liten LS87</v>
-      </c>
-      <c r="AS397">
-        <v>0</v>
-      </c>
-      <c r="AT397">
-        <v>0</v>
-      </c>
-      <c r="AU397">
-        <v>0</v>
-      </c>
-      <c r="AV397">
-        <v>0</v>
-      </c>
-      <c r="AW397">
-        <v>0</v>
-      </c>
-      <c r="AX397">
-        <v>0</v>
-      </c>
-      <c r="AY397">
-        <v>0</v>
-      </c>
-      <c r="AZ397">
-        <v>0</v>
-      </c>
-      <c r="BA397">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="398">
-      <c r="A398" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="B398" t="str">
-        <v>TBD</v>
-      </c>
-      <c r="C398" t="str">
-        <v>Drylock</v>
-      </c>
-      <c r="D398" t="str">
-        <v>CZ11</v>
-      </c>
-      <c r="E398" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="F398" t="str">
-        <v>hygiene</v>
-      </c>
-      <c r="G398" t="str">
-        <v>TS</v>
-      </c>
-      <c r="H398" t="str">
-        <v>S</v>
-      </c>
-      <c r="I398" t="str">
-        <v>Mono</v>
-      </c>
-      <c r="J398" t="str">
-        <v>G08 - honeycombs</v>
-      </c>
-      <c r="K398">
-        <v>12</v>
-      </c>
-      <c r="L398">
-        <v>0</v>
-      </c>
-      <c r="M398" t="str">
-        <v>hydrophilic+Aloe+vitE</v>
-      </c>
-      <c r="N398" t="str">
-        <v>100 - white</v>
-      </c>
-      <c r="O398" t="str">
-        <v>Svobodova</v>
-      </c>
-      <c r="P398">
-        <v>0.8423076923076923</v>
-      </c>
-      <c r="Q398">
-        <v>1169.28</v>
-      </c>
-      <c r="R398">
-        <v>1.0153381669678316</v>
-      </c>
-      <c r="S398">
-        <v>0.08</v>
-      </c>
-      <c r="T398">
-        <v>0.05</v>
-      </c>
-      <c r="U398">
-        <v>0.996</v>
-      </c>
-      <c r="V398">
-        <v>0.866</v>
-      </c>
-      <c r="W398">
-        <v>0</v>
-      </c>
-      <c r="X398">
-        <v>0</v>
-      </c>
-      <c r="Y398">
-        <v>0</v>
-      </c>
-      <c r="Z398">
-        <v>0</v>
-      </c>
-      <c r="AA398">
-        <v>0</v>
-      </c>
-      <c r="AB398">
-        <v>0</v>
-      </c>
-      <c r="AC398">
-        <v>0.005208333333333334</v>
-      </c>
-      <c r="AD398">
-        <v>0.00005</v>
-      </c>
-      <c r="AE398">
-        <v>0.0001</v>
-      </c>
-      <c r="AF398">
-        <v>0.004</v>
-      </c>
-      <c r="AG398">
-        <v>0</v>
-      </c>
-      <c r="AH398">
-        <v>0</v>
-      </c>
-      <c r="AI398">
-        <v>0</v>
-      </c>
-      <c r="AJ398">
-        <v>0</v>
-      </c>
-      <c r="AK398">
-        <v>1.0053583333333336</v>
-      </c>
-      <c r="AL398" t="str">
-        <v>S: PPSB - Mosten NB 425</v>
-      </c>
-      <c r="AM398">
-        <v>0</v>
-      </c>
-      <c r="AN398">
-        <v>0</v>
-      </c>
-      <c r="AO398">
-        <v>0</v>
-      </c>
-      <c r="AS398" t="str">
-        <v>S: Zušl. - Silastol PHP 207</v>
-      </c>
-      <c r="AT398" t="str">
-        <v>Aloe Vera - powder 200x</v>
-      </c>
-      <c r="AU398" t="str">
-        <v>Silastol Care T- Vitamine E</v>
-      </c>
-      <c r="AV398" t="str">
-        <v>S: Pig.  - CC10084467BG bílá 60%</v>
-      </c>
-      <c r="AW398">
-        <v>0</v>
-      </c>
-      <c r="AX398">
-        <v>0</v>
-      </c>
-      <c r="AY398">
-        <v>0</v>
-      </c>
-      <c r="AZ398">
-        <v>0</v>
-      </c>
-      <c r="BA398">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BA398"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BA392"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>